<commit_message>
Added 1nF MLCCs to database
</commit_message>
<xml_diff>
--- a/To Add v2/Capacitors - Unpolarized.xlsx
+++ b/To Add v2/Capacitors - Unpolarized.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\To Add v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC629D8D-8F4D-4190-AE01-ED899AFE5AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6E17BC-CCAB-43EA-8519-13C29E585784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2184" yWindow="228" windowWidth="18732" windowHeight="11508" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="194">
   <si>
     <t>Totals</t>
   </si>
@@ -576,6 +576,48 @@
   </si>
   <si>
     <t>https://product.tdk.com/en/system/files/dam/doc/product/capacitor/ceramic/mlcc/catalog/mlcc_automotive_midvoltage_en.pdf</t>
+  </si>
+  <si>
+    <t>1n</t>
+  </si>
+  <si>
+    <t>GRM1555C1H102JA01D</t>
+  </si>
+  <si>
+    <t>490-3244-1-ND</t>
+  </si>
+  <si>
+    <t>https://search.murata.co.jp/Ceramy/image/img/A01X/G101/ENG/GRM1555C1H102JA01-01.pdf</t>
+  </si>
+  <si>
+    <t>GRM1885C1H102JA01D</t>
+  </si>
+  <si>
+    <t>490-1451-1-ND</t>
+  </si>
+  <si>
+    <t>https://search.murata.co.jp/Ceramy/image/img/A01X/G101/ENG/GRM1885C1H102JA01-01.pdf</t>
+  </si>
+  <si>
+    <t>GCM188R71H102KA37D</t>
+  </si>
+  <si>
+    <t>490-4777-1-ND</t>
+  </si>
+  <si>
+    <t>https://search.murata.co.jp/Ceramy/image/img/A01X/G101/ENG/GCM188R71H102KA37-01.pdf</t>
+  </si>
+  <si>
+    <t>CL21B102KCANNNC</t>
+  </si>
+  <si>
+    <t>1276-1169-1-ND</t>
+  </si>
+  <si>
+    <t>CL31B102KBCNNNC</t>
+  </si>
+  <si>
+    <t>1276-1050-1-ND</t>
   </si>
 </sst>
 </file>
@@ -967,104 +1009,104 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB95"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="36.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" customWidth="1"/>
+    <col min="3" max="3" width="36.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.08984375" customWidth="1"/>
+    <col min="7" max="7" width="10.08984375" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="12.21875" customWidth="1"/>
+    <col min="10" max="10" width="12.1796875" customWidth="1"/>
     <col min="11" max="11" width="24" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5546875" customWidth="1"/>
-    <col min="14" max="14" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.21875" customWidth="1"/>
-    <col min="17" max="17" width="22.33203125" customWidth="1"/>
-    <col min="18" max="18" width="10.88671875" customWidth="1"/>
-    <col min="19" max="19" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" customWidth="1"/>
+    <col min="14" max="14" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.1796875" customWidth="1"/>
+    <col min="17" max="17" width="22.36328125" customWidth="1"/>
+    <col min="18" max="18" width="10.90625" customWidth="1"/>
+    <col min="19" max="19" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="B1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2">
         <f t="shared" ref="C2:T2" si="0">COUNTA(C7:C10007)</f>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="G2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="H2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="I2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="K2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="L2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="Q2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="S2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="T2">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="AA2" t="s">
         <v>1</v>
@@ -1074,16 +1116,16 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="AA3" t="s">
         <v>2</v>
       </c>
       <c r="AB3">
         <f>MAX(C2:R2)</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1146,10 +1188,10 @@
       </c>
       <c r="AB4">
         <f>SUM(Y7:Y9999)</f>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
       <c r="AA5" t="s">
         <v>5</v>
       </c>
@@ -1158,7 +1200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>6</v>
       </c>
@@ -1223,7 +1265,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1302,7 +1344,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1374,7 +1416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1446,7 +1488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>4</v>
       </c>
@@ -1518,7 +1560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>5</v>
       </c>
@@ -1590,7 +1632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>6</v>
       </c>
@@ -1662,7 +1704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>7</v>
       </c>
@@ -1734,12 +1776,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>8</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" ref="C14:C44" si="5">_xlfn.CONCAT(D14,"F ",F14,"V ",E14," ",G14," ",I14," ",J14," ",R14)</f>
+        <f t="shared" ref="C14:C49" si="5">_xlfn.CONCAT(D14,"F ",F14,"V ",E14," ",G14," ",I14," ",J14," ",R14)</f>
         <v>10nF 35V 0402 C0G SMD MLCC  </v>
       </c>
       <c r="D14" t="s">
@@ -1806,7 +1848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>9</v>
       </c>
@@ -1878,7 +1920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>10</v>
       </c>
@@ -1950,7 +1992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>11</v>
       </c>
@@ -2022,7 +2064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>12</v>
       </c>
@@ -2094,7 +2136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>13</v>
       </c>
@@ -2166,7 +2208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>14</v>
       </c>
@@ -2238,7 +2280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>15</v>
       </c>
@@ -2310,7 +2352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>16</v>
       </c>
@@ -2382,7 +2424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>17</v>
       </c>
@@ -2454,7 +2496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>18</v>
       </c>
@@ -2526,7 +2568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>19</v>
       </c>
@@ -2598,7 +2640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>20</v>
       </c>
@@ -2670,7 +2712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>21</v>
       </c>
@@ -2742,7 +2784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>22</v>
       </c>
@@ -2814,7 +2856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>23</v>
       </c>
@@ -2886,7 +2928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>24</v>
       </c>
@@ -2958,7 +3000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>25</v>
       </c>
@@ -3030,7 +3072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>26</v>
       </c>
@@ -3102,7 +3144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>27</v>
       </c>
@@ -3174,7 +3216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>28</v>
       </c>
@@ -3246,7 +3288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>29</v>
       </c>
@@ -3306,19 +3348,19 @@
         <v>1</v>
       </c>
       <c r="W35">
-        <f t="shared" ref="W35" si="17">COUNTBLANK(C35:R35)</f>
+        <f t="shared" ref="W35:W40" si="17">COUNTBLANK(C35:R35)</f>
         <v>0</v>
       </c>
       <c r="X35">
-        <f t="shared" ref="X35" si="18">100*COUNTA(C35:R35)/$AB$7</f>
+        <f t="shared" ref="X35:X40" si="18">100*COUNTA(C35:R35)/$AB$7</f>
         <v>100</v>
       </c>
       <c r="Y35">
-        <f t="shared" ref="Y35" si="19">IF(X35=100,1,0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.3">
+        <f t="shared" ref="Y35:Y40" si="19">IF(X35=100,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>30</v>
       </c>
@@ -3377,8 +3419,20 @@
       <c r="T36" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="W36">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="X36">
+        <f t="shared" si="18"/>
+        <v>100</v>
+      </c>
+      <c r="Y36">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>31</v>
       </c>
@@ -3437,8 +3491,20 @@
       <c r="T37" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="W37">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="X37">
+        <f t="shared" si="18"/>
+        <v>100</v>
+      </c>
+      <c r="Y37">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>32</v>
       </c>
@@ -3497,8 +3563,20 @@
       <c r="T38" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="W38">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="X38">
+        <f t="shared" si="18"/>
+        <v>100</v>
+      </c>
+      <c r="Y38">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>33</v>
       </c>
@@ -3557,8 +3635,20 @@
       <c r="T39" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="W39">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="X39">
+        <f t="shared" si="18"/>
+        <v>100</v>
+      </c>
+      <c r="Y39">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>34</v>
       </c>
@@ -3617,8 +3707,20 @@
       <c r="T40" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="W40">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="X40">
+        <f t="shared" si="18"/>
+        <v>100</v>
+      </c>
+      <c r="Y40">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>35</v>
       </c>
@@ -3677,8 +3779,20 @@
       <c r="T41" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="W41">
+        <f t="shared" ref="W41:W49" si="20">COUNTBLANK(C41:R41)</f>
+        <v>0</v>
+      </c>
+      <c r="X41">
+        <f t="shared" ref="X41:X49" si="21">100*COUNTA(C41:R41)/$AB$7</f>
+        <v>100</v>
+      </c>
+      <c r="Y41">
+        <f t="shared" ref="Y41:Y49" si="22">IF(X41=100,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>36</v>
       </c>
@@ -3737,8 +3851,20 @@
       <c r="T42" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="W42">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X42">
+        <f t="shared" si="21"/>
+        <v>100</v>
+      </c>
+      <c r="Y42">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>37</v>
       </c>
@@ -3797,8 +3923,20 @@
       <c r="T43" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="W43">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X43">
+        <f t="shared" si="21"/>
+        <v>100</v>
+      </c>
+      <c r="Y43">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>38</v>
       </c>
@@ -3857,158 +3995,515 @@
       <c r="T44" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="E45" s="2"/>
-    </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="E46" s="2"/>
-    </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="E47" s="2"/>
-    </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="E48" s="2"/>
-    </row>
-    <row r="49" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E49" s="2"/>
-    </row>
-    <row r="50" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="W44">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X44">
+        <f t="shared" si="21"/>
+        <v>100</v>
+      </c>
+      <c r="Y44">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>49</v>
+      </c>
+      <c r="C45" t="str">
+        <f t="shared" si="5"/>
+        <v>1nF 50V 0402 C0G SMD MLCC  </v>
+      </c>
+      <c r="D45" t="s">
+        <v>180</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F45">
+        <v>50</v>
+      </c>
+      <c r="G45" t="s">
+        <v>98</v>
+      </c>
+      <c r="H45">
+        <v>5</v>
+      </c>
+      <c r="I45" t="s">
+        <v>28</v>
+      </c>
+      <c r="J45" t="s">
+        <v>29</v>
+      </c>
+      <c r="K45" t="s">
+        <v>57</v>
+      </c>
+      <c r="L45" t="s">
+        <v>181</v>
+      </c>
+      <c r="M45" t="s">
+        <v>37</v>
+      </c>
+      <c r="N45" t="s">
+        <v>182</v>
+      </c>
+      <c r="O45" t="s">
+        <v>183</v>
+      </c>
+      <c r="P45" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>173</v>
+      </c>
+      <c r="R45" t="s">
+        <v>42</v>
+      </c>
+      <c r="S45" t="b">
+        <v>0</v>
+      </c>
+      <c r="T45" t="b">
+        <v>1</v>
+      </c>
+      <c r="W45">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X45">
+        <f t="shared" si="21"/>
+        <v>100</v>
+      </c>
+      <c r="Y45">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>40</v>
+      </c>
+      <c r="C46" t="str">
+        <f t="shared" si="5"/>
+        <v>1nF 50V 0603 C0G SMD MLCC  </v>
+      </c>
+      <c r="D46" t="s">
+        <v>180</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F46">
+        <v>50</v>
+      </c>
+      <c r="G46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H46">
+        <v>5</v>
+      </c>
+      <c r="I46" t="s">
+        <v>28</v>
+      </c>
+      <c r="J46" t="s">
+        <v>29</v>
+      </c>
+      <c r="K46" t="s">
+        <v>57</v>
+      </c>
+      <c r="L46" t="s">
+        <v>184</v>
+      </c>
+      <c r="M46" t="s">
+        <v>37</v>
+      </c>
+      <c r="N46" t="s">
+        <v>185</v>
+      </c>
+      <c r="O46" t="s">
+        <v>186</v>
+      </c>
+      <c r="P46" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>41</v>
+      </c>
+      <c r="R46" t="s">
+        <v>42</v>
+      </c>
+      <c r="S46" t="b">
+        <v>0</v>
+      </c>
+      <c r="T46" t="b">
+        <v>1</v>
+      </c>
+      <c r="W46">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X46">
+        <f t="shared" si="21"/>
+        <v>100</v>
+      </c>
+      <c r="Y46">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>41</v>
+      </c>
+      <c r="C47" t="str">
+        <f t="shared" si="5"/>
+        <v>1nF 50V 0603 X7R SMD MLCC Automotive</v>
+      </c>
+      <c r="D47" t="s">
+        <v>180</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F47">
+        <v>50</v>
+      </c>
+      <c r="G47" t="s">
+        <v>33</v>
+      </c>
+      <c r="H47">
+        <v>10</v>
+      </c>
+      <c r="I47" t="s">
+        <v>28</v>
+      </c>
+      <c r="J47" t="s">
+        <v>29</v>
+      </c>
+      <c r="K47" t="s">
+        <v>57</v>
+      </c>
+      <c r="L47" t="s">
+        <v>187</v>
+      </c>
+      <c r="M47" t="s">
+        <v>37</v>
+      </c>
+      <c r="N47" t="s">
+        <v>188</v>
+      </c>
+      <c r="O47" t="s">
+        <v>189</v>
+      </c>
+      <c r="P47" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>41</v>
+      </c>
+      <c r="R47" t="s">
+        <v>100</v>
+      </c>
+      <c r="S47" t="b">
+        <v>0</v>
+      </c>
+      <c r="T47" t="b">
+        <v>1</v>
+      </c>
+      <c r="W47">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X47">
+        <f t="shared" si="21"/>
+        <v>100</v>
+      </c>
+      <c r="Y47">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>42</v>
+      </c>
+      <c r="C48" t="str">
+        <f t="shared" si="5"/>
+        <v>1nF 100V 0805 X7R SMD MLCC  </v>
+      </c>
+      <c r="D48" t="s">
+        <v>180</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F48">
+        <v>100</v>
+      </c>
+      <c r="G48" t="s">
+        <v>33</v>
+      </c>
+      <c r="H48">
+        <v>10</v>
+      </c>
+      <c r="I48" t="s">
+        <v>28</v>
+      </c>
+      <c r="J48" t="s">
+        <v>29</v>
+      </c>
+      <c r="K48" t="s">
+        <v>53</v>
+      </c>
+      <c r="L48" t="s">
+        <v>190</v>
+      </c>
+      <c r="M48" t="s">
+        <v>37</v>
+      </c>
+      <c r="N48" t="s">
+        <v>191</v>
+      </c>
+      <c r="O48" t="s">
+        <v>90</v>
+      </c>
+      <c r="P48" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>95</v>
+      </c>
+      <c r="R48" t="s">
+        <v>42</v>
+      </c>
+      <c r="S48" t="b">
+        <v>0</v>
+      </c>
+      <c r="T48" t="b">
+        <v>1</v>
+      </c>
+      <c r="W48">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X48">
+        <f t="shared" si="21"/>
+        <v>100</v>
+      </c>
+      <c r="Y48">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>43</v>
+      </c>
+      <c r="C49" t="str">
+        <f t="shared" si="5"/>
+        <v>1nF 50V 1206 X7R SMD MLCC  </v>
+      </c>
+      <c r="D49" t="s">
+        <v>180</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F49">
+        <v>50</v>
+      </c>
+      <c r="G49" t="s">
+        <v>33</v>
+      </c>
+      <c r="H49">
+        <v>10</v>
+      </c>
+      <c r="I49" t="s">
+        <v>28</v>
+      </c>
+      <c r="J49" t="s">
+        <v>29</v>
+      </c>
+      <c r="K49" t="s">
+        <v>53</v>
+      </c>
+      <c r="L49" t="s">
+        <v>192</v>
+      </c>
+      <c r="M49" t="s">
+        <v>37</v>
+      </c>
+      <c r="N49" t="s">
+        <v>193</v>
+      </c>
+      <c r="O49" t="s">
+        <v>90</v>
+      </c>
+      <c r="P49" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>52</v>
+      </c>
+      <c r="R49" t="s">
+        <v>42</v>
+      </c>
+      <c r="S49" t="b">
+        <v>0</v>
+      </c>
+      <c r="T49" t="b">
+        <v>1</v>
+      </c>
+      <c r="W49">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="X49">
+        <f t="shared" si="21"/>
+        <v>100</v>
+      </c>
+      <c r="Y49">
+        <f t="shared" si="22"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E50" s="2"/>
     </row>
-    <row r="51" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E51" s="2"/>
     </row>
-    <row r="52" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E52" s="2"/>
     </row>
-    <row r="53" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E53" s="2"/>
     </row>
-    <row r="54" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E54" s="2"/>
     </row>
-    <row r="55" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E55" s="2"/>
     </row>
-    <row r="56" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E56" s="2"/>
     </row>
-    <row r="57" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E57" s="2"/>
     </row>
-    <row r="58" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E58" s="2"/>
     </row>
-    <row r="59" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E59" s="2"/>
     </row>
-    <row r="60" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E60" s="2"/>
     </row>
-    <row r="61" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E61" s="2"/>
     </row>
-    <row r="62" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E62" s="2"/>
     </row>
-    <row r="63" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E63" s="2"/>
     </row>
-    <row r="64" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E64" s="2"/>
     </row>
-    <row r="65" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E65" s="2"/>
     </row>
-    <row r="66" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E66" s="2"/>
     </row>
-    <row r="67" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E67" s="2"/>
     </row>
-    <row r="68" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E68" s="2"/>
     </row>
-    <row r="69" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E69" s="2"/>
     </row>
-    <row r="70" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E70" s="2"/>
     </row>
-    <row r="71" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E71" s="2"/>
     </row>
-    <row r="72" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E72" s="2"/>
     </row>
-    <row r="73" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E73" s="2"/>
     </row>
-    <row r="74" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E74" s="2"/>
     </row>
-    <row r="75" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E75" s="2"/>
     </row>
-    <row r="76" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E76" s="2"/>
     </row>
-    <row r="77" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E77" s="2"/>
     </row>
-    <row r="78" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E78" s="2"/>
     </row>
-    <row r="79" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E79" s="2"/>
     </row>
-    <row r="80" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E80" s="2"/>
     </row>
-    <row r="81" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E81" s="2"/>
     </row>
-    <row r="82" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E82" s="2"/>
     </row>
-    <row r="83" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E83" s="2"/>
     </row>
-    <row r="84" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E84" s="2"/>
     </row>
-    <row r="85" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E85" s="2"/>
     </row>
-    <row r="86" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E86" s="2"/>
     </row>
-    <row r="87" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E87" s="2"/>
     </row>
-    <row r="88" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="88" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E88" s="2"/>
     </row>
-    <row r="89" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="89" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E89" s="2"/>
     </row>
-    <row r="90" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="90" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E90" s="2"/>
     </row>
-    <row r="91" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E91" s="2"/>
     </row>
-    <row r="92" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="92" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E92" s="2"/>
     </row>
-    <row r="93" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="93" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E93" s="2"/>
     </row>
-    <row r="94" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="94" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E94" s="2"/>
     </row>
-    <row r="95" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="95" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E95" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added some 4.7nF X7R MLCCs
</commit_message>
<xml_diff>
--- a/To Add v2/Capacitors - Unpolarized.xlsx
+++ b/To Add v2/Capacitors - Unpolarized.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6E17BC-CCAB-43EA-8519-13C29E585784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065457B4-892A-43E7-B839-6D8A3AB08B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="202">
   <si>
     <t>Totals</t>
   </si>
@@ -618,6 +618,30 @@
   </si>
   <si>
     <t>1276-1050-1-ND</t>
+  </si>
+  <si>
+    <t>4.7n</t>
+  </si>
+  <si>
+    <t>407n</t>
+  </si>
+  <si>
+    <t>CGA3E2X7R1H472K080AA</t>
+  </si>
+  <si>
+    <t>445-5661-1-ND</t>
+  </si>
+  <si>
+    <t>https://product.tdk.com/system/files/dam/doc/product/capacitor/ceramic/mlcc/catalog/mlcc_automotive_general_en.pdf</t>
+  </si>
+  <si>
+    <t>CL21B472KBANNNC</t>
+  </si>
+  <si>
+    <t>1276-1155-1-ND</t>
+  </si>
+  <si>
+    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/1169/CL21B472KBANNNE_Spec.pdf</t>
   </si>
 </sst>
 </file>
@@ -1038,75 +1062,75 @@
       </c>
       <c r="C2">
         <f t="shared" ref="C2:T2" si="0">COUNTA(C7:C10007)</f>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="Q2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="S2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="T2">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="AA2" t="s">
         <v>1</v>
@@ -1122,7 +1146,7 @@
       </c>
       <c r="AB3">
         <f>MAX(C2:R2)</f>
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.35">
@@ -1188,7 +1212,7 @@
       </c>
       <c r="AB4">
         <f>SUM(Y7:Y9999)</f>
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.35">
@@ -1781,7 +1805,7 @@
         <v>8</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" ref="C14:C49" si="5">_xlfn.CONCAT(D14,"F ",F14,"V ",E14," ",G14," ",I14," ",J14," ",R14)</f>
+        <f t="shared" ref="C14:C51" si="5">_xlfn.CONCAT(D14,"F ",F14,"V ",E14," ",G14," ",I14," ",J14," ",R14)</f>
         <v>10nF 35V 0402 C0G SMD MLCC  </v>
       </c>
       <c r="D14" t="s">
@@ -4369,10 +4393,148 @@
       </c>
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E50" s="2"/>
+      <c r="A50">
+        <v>44</v>
+      </c>
+      <c r="C50" t="str">
+        <f t="shared" si="5"/>
+        <v>4.7nF 50V 0603 X7R SMD MLCC Automotive</v>
+      </c>
+      <c r="D50" t="s">
+        <v>194</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F50">
+        <v>50</v>
+      </c>
+      <c r="G50" t="s">
+        <v>33</v>
+      </c>
+      <c r="H50">
+        <v>10</v>
+      </c>
+      <c r="I50" t="s">
+        <v>28</v>
+      </c>
+      <c r="J50" t="s">
+        <v>29</v>
+      </c>
+      <c r="K50" t="s">
+        <v>105</v>
+      </c>
+      <c r="L50" t="s">
+        <v>196</v>
+      </c>
+      <c r="M50" t="s">
+        <v>37</v>
+      </c>
+      <c r="N50" t="s">
+        <v>197</v>
+      </c>
+      <c r="O50" t="s">
+        <v>198</v>
+      </c>
+      <c r="P50" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>41</v>
+      </c>
+      <c r="R50" t="s">
+        <v>100</v>
+      </c>
+      <c r="S50" t="b">
+        <v>0</v>
+      </c>
+      <c r="T50" t="b">
+        <v>1</v>
+      </c>
+      <c r="W50">
+        <f t="shared" ref="W50:W51" si="23">COUNTBLANK(C50:R50)</f>
+        <v>0</v>
+      </c>
+      <c r="X50">
+        <f t="shared" ref="X50:X51" si="24">100*COUNTA(C50:R50)/$AB$7</f>
+        <v>100</v>
+      </c>
+      <c r="Y50">
+        <f t="shared" ref="Y50:Y51" si="25">IF(X50=100,1,0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E51" s="2"/>
+      <c r="A51">
+        <v>45</v>
+      </c>
+      <c r="C51" t="str">
+        <f t="shared" si="5"/>
+        <v>407nF 50V 0805 X7R SMD MLCC  </v>
+      </c>
+      <c r="D51" t="s">
+        <v>195</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F51">
+        <v>50</v>
+      </c>
+      <c r="G51" t="s">
+        <v>33</v>
+      </c>
+      <c r="H51">
+        <v>10</v>
+      </c>
+      <c r="I51" t="s">
+        <v>28</v>
+      </c>
+      <c r="J51" t="s">
+        <v>29</v>
+      </c>
+      <c r="K51" t="s">
+        <v>53</v>
+      </c>
+      <c r="L51" t="s">
+        <v>199</v>
+      </c>
+      <c r="M51" t="s">
+        <v>37</v>
+      </c>
+      <c r="N51" t="s">
+        <v>200</v>
+      </c>
+      <c r="O51" t="s">
+        <v>201</v>
+      </c>
+      <c r="P51" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>95</v>
+      </c>
+      <c r="R51" t="s">
+        <v>42</v>
+      </c>
+      <c r="S51" t="b">
+        <v>0</v>
+      </c>
+      <c r="T51" t="b">
+        <v>1</v>
+      </c>
+      <c r="W51">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="X51">
+        <f t="shared" si="24"/>
+        <v>100</v>
+      </c>
+      <c r="Y51">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E52" s="2"/>

</xml_diff>

<commit_message>
Corrected capacitance in a MLCC
</commit_message>
<xml_diff>
--- a/To Add v2/Capacitors - Unpolarized.xlsx
+++ b/To Add v2/Capacitors - Unpolarized.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065457B4-892A-43E7-B839-6D8A3AB08B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A407A8-592F-4682-8000-D1D714BE0311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="201">
   <si>
     <t>Totals</t>
   </si>
@@ -621,9 +621,6 @@
   </si>
   <si>
     <t>4.7n</t>
-  </si>
-  <si>
-    <t>407n</t>
   </si>
   <si>
     <t>CGA3E2X7R1H472K080AA</t>
@@ -4425,16 +4422,16 @@
         <v>105</v>
       </c>
       <c r="L50" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M50" t="s">
         <v>37</v>
       </c>
       <c r="N50" t="s">
+        <v>196</v>
+      </c>
+      <c r="O50" t="s">
         <v>197</v>
-      </c>
-      <c r="O50" t="s">
-        <v>198</v>
       </c>
       <c r="P50" t="s">
         <v>40</v>
@@ -4470,10 +4467,10 @@
       </c>
       <c r="C51" t="str">
         <f t="shared" si="5"/>
-        <v>407nF 50V 0805 X7R SMD MLCC  </v>
+        <v>4.7nF 50V 0805 X7R SMD MLCC  </v>
       </c>
       <c r="D51" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>79</v>
@@ -4497,16 +4494,16 @@
         <v>53</v>
       </c>
       <c r="L51" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="M51" t="s">
         <v>37</v>
       </c>
       <c r="N51" t="s">
+        <v>199</v>
+      </c>
+      <c r="O51" t="s">
         <v>200</v>
-      </c>
-      <c r="O51" t="s">
-        <v>201</v>
       </c>
       <c r="P51" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Added 4.7nF C0G MLCCs and a 100nF X7R 0603
</commit_message>
<xml_diff>
--- a/To Add v2/Capacitors - Unpolarized.xlsx
+++ b/To Add v2/Capacitors - Unpolarized.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A407A8-592F-4682-8000-D1D714BE0311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381FF984-DD05-48EE-B0C2-33525A4F8A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="213">
   <si>
     <t>Totals</t>
   </si>
@@ -639,6 +639,42 @@
   </si>
   <si>
     <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/1169/CL21B472KBANNNE_Spec.pdf</t>
+  </si>
+  <si>
+    <t>GCM188R71H104KA57J</t>
+  </si>
+  <si>
+    <t>490-8020-1-ND</t>
+  </si>
+  <si>
+    <t>https://search.murata.co.jp/Ceramy/image/img/A01X/G101/ENG/GCM188R71H104KA57-01.pdf</t>
+  </si>
+  <si>
+    <t>GRM1885C1H472JA01D</t>
+  </si>
+  <si>
+    <t>490-9669-1-ND</t>
+  </si>
+  <si>
+    <t>https://search.murata.co.jp/Ceramy/image/img/A01X/G101/ENG/GRM1885C1H472JA01-01.pdf</t>
+  </si>
+  <si>
+    <t>GRM2165C1H472JA01D</t>
+  </si>
+  <si>
+    <t>490-3044-1-ND</t>
+  </si>
+  <si>
+    <t>https://search.murata.co.jp/Ceramy/image/img/A01X/G101/ENG/GRM2165C1H472JA01-01.pdf</t>
+  </si>
+  <si>
+    <t>C3216C0G2E472J115AA</t>
+  </si>
+  <si>
+    <t>445-2333-1-ND</t>
+  </si>
+  <si>
+    <t>https://product.tdk.com/system/files/dam/doc/product/capacitor/ceramic/mlcc/catalog/mlcc_commercial_midvoltage_en.pdf</t>
   </si>
 </sst>
 </file>
@@ -1059,75 +1095,75 @@
       </c>
       <c r="C2">
         <f t="shared" ref="C2:T2" si="0">COUNTA(C7:C10007)</f>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="H2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="I2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="L2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="Q2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="S2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="T2">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="AA2" t="s">
         <v>1</v>
@@ -1143,7 +1179,7 @@
       </c>
       <c r="AB3">
         <f>MAX(C2:R2)</f>
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.35">
@@ -1209,7 +1245,7 @@
       </c>
       <c r="AB4">
         <f>SUM(Y7:Y9999)</f>
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.35">
@@ -1802,7 +1838,7 @@
         <v>8</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" ref="C14:C51" si="5">_xlfn.CONCAT(D14,"F ",F14,"V ",E14," ",G14," ",I14," ",J14," ",R14)</f>
+        <f t="shared" ref="C14:C55" si="5">_xlfn.CONCAT(D14,"F ",F14,"V ",E14," ",G14," ",I14," ",J14," ",R14)</f>
         <v>10nF 35V 0402 C0G SMD MLCC  </v>
       </c>
       <c r="D14" t="s">
@@ -4449,15 +4485,15 @@
         <v>1</v>
       </c>
       <c r="W50">
-        <f t="shared" ref="W50:W51" si="23">COUNTBLANK(C50:R50)</f>
+        <f t="shared" ref="W50:W55" si="23">COUNTBLANK(C50:R50)</f>
         <v>0</v>
       </c>
       <c r="X50">
-        <f t="shared" ref="X50:X51" si="24">100*COUNTA(C50:R50)/$AB$7</f>
+        <f t="shared" ref="X50:X55" si="24">100*COUNTA(C50:R50)/$AB$7</f>
         <v>100</v>
       </c>
       <c r="Y50">
-        <f t="shared" ref="Y50:Y51" si="25">IF(X50=100,1,0)</f>
+        <f t="shared" ref="Y50:Y55" si="25">IF(X50=100,1,0)</f>
         <v>1</v>
       </c>
     </row>
@@ -4534,16 +4570,292 @@
       </c>
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E52" s="2"/>
+      <c r="A52">
+        <v>46</v>
+      </c>
+      <c r="C52" t="str">
+        <f t="shared" si="5"/>
+        <v>100nF 50V 0603 X7R SMD MLCC Automotive</v>
+      </c>
+      <c r="D52" t="s">
+        <v>64</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F52">
+        <v>50</v>
+      </c>
+      <c r="G52" t="s">
+        <v>33</v>
+      </c>
+      <c r="H52">
+        <v>10</v>
+      </c>
+      <c r="I52" t="s">
+        <v>28</v>
+      </c>
+      <c r="J52" t="s">
+        <v>29</v>
+      </c>
+      <c r="K52" t="s">
+        <v>57</v>
+      </c>
+      <c r="L52" t="s">
+        <v>201</v>
+      </c>
+      <c r="M52" t="s">
+        <v>37</v>
+      </c>
+      <c r="N52" t="s">
+        <v>202</v>
+      </c>
+      <c r="O52" t="s">
+        <v>203</v>
+      </c>
+      <c r="P52" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>41</v>
+      </c>
+      <c r="R52" t="s">
+        <v>100</v>
+      </c>
+      <c r="S52" t="b">
+        <v>0</v>
+      </c>
+      <c r="T52" t="b">
+        <v>1</v>
+      </c>
+      <c r="W52">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="X52">
+        <f t="shared" si="24"/>
+        <v>100</v>
+      </c>
+      <c r="Y52">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E53" s="2"/>
+      <c r="A53">
+        <v>47</v>
+      </c>
+      <c r="C53" t="str">
+        <f t="shared" si="5"/>
+        <v>4.7nF 50V 0603 C0G SMD MLCC  </v>
+      </c>
+      <c r="D53" t="s">
+        <v>194</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F53">
+        <v>50</v>
+      </c>
+      <c r="G53" t="s">
+        <v>98</v>
+      </c>
+      <c r="H53">
+        <v>5</v>
+      </c>
+      <c r="I53" t="s">
+        <v>28</v>
+      </c>
+      <c r="J53" t="s">
+        <v>29</v>
+      </c>
+      <c r="K53" t="s">
+        <v>57</v>
+      </c>
+      <c r="L53" t="s">
+        <v>204</v>
+      </c>
+      <c r="M53" t="s">
+        <v>37</v>
+      </c>
+      <c r="N53" t="s">
+        <v>205</v>
+      </c>
+      <c r="O53" t="s">
+        <v>206</v>
+      </c>
+      <c r="P53" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>41</v>
+      </c>
+      <c r="R53" t="s">
+        <v>42</v>
+      </c>
+      <c r="S53" t="b">
+        <v>0</v>
+      </c>
+      <c r="T53" t="b">
+        <v>1</v>
+      </c>
+      <c r="W53">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="X53">
+        <f t="shared" si="24"/>
+        <v>100</v>
+      </c>
+      <c r="Y53">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E54" s="2"/>
+      <c r="A54">
+        <v>48</v>
+      </c>
+      <c r="C54" t="str">
+        <f t="shared" si="5"/>
+        <v>4.7nF 50V 0805 C0G SMD MLCC  </v>
+      </c>
+      <c r="D54" t="s">
+        <v>194</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F54">
+        <v>50</v>
+      </c>
+      <c r="G54" t="s">
+        <v>98</v>
+      </c>
+      <c r="H54">
+        <v>5</v>
+      </c>
+      <c r="I54" t="s">
+        <v>28</v>
+      </c>
+      <c r="J54" t="s">
+        <v>29</v>
+      </c>
+      <c r="K54" t="s">
+        <v>57</v>
+      </c>
+      <c r="L54" t="s">
+        <v>207</v>
+      </c>
+      <c r="M54" t="s">
+        <v>37</v>
+      </c>
+      <c r="N54" t="s">
+        <v>208</v>
+      </c>
+      <c r="O54" t="s">
+        <v>209</v>
+      </c>
+      <c r="P54" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>95</v>
+      </c>
+      <c r="R54" t="s">
+        <v>42</v>
+      </c>
+      <c r="S54" t="b">
+        <v>0</v>
+      </c>
+      <c r="T54" t="b">
+        <v>1</v>
+      </c>
+      <c r="W54">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="X54">
+        <f t="shared" si="24"/>
+        <v>100</v>
+      </c>
+      <c r="Y54">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E55" s="2"/>
+      <c r="A55">
+        <v>49</v>
+      </c>
+      <c r="C55" t="str">
+        <f t="shared" si="5"/>
+        <v>4.7nF 250V 1206 C0G SMD MLCC  </v>
+      </c>
+      <c r="D55" t="s">
+        <v>194</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F55">
+        <v>250</v>
+      </c>
+      <c r="G55" t="s">
+        <v>98</v>
+      </c>
+      <c r="H55">
+        <v>5</v>
+      </c>
+      <c r="I55" t="s">
+        <v>28</v>
+      </c>
+      <c r="J55" t="s">
+        <v>29</v>
+      </c>
+      <c r="K55" t="s">
+        <v>105</v>
+      </c>
+      <c r="L55" t="s">
+        <v>210</v>
+      </c>
+      <c r="M55" t="s">
+        <v>37</v>
+      </c>
+      <c r="N55" t="s">
+        <v>211</v>
+      </c>
+      <c r="O55" t="s">
+        <v>212</v>
+      </c>
+      <c r="P55" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>52</v>
+      </c>
+      <c r="R55" t="s">
+        <v>42</v>
+      </c>
+      <c r="S55" t="b">
+        <v>0</v>
+      </c>
+      <c r="T55" t="b">
+        <v>1</v>
+      </c>
+      <c r="W55">
+        <f t="shared" si="23"/>
+        <v>0</v>
+      </c>
+      <c r="X55">
+        <f t="shared" si="24"/>
+        <v>100</v>
+      </c>
+      <c r="Y55">
+        <f t="shared" si="25"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E56" s="2"/>

</xml_diff>

<commit_message>
Added 220nF X7R MLCCs in 0603, 0805, and 1206 sizes
</commit_message>
<xml_diff>
--- a/To Add v2/Capacitors - Unpolarized.xlsx
+++ b/To Add v2/Capacitors - Unpolarized.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381FF984-DD05-48EE-B0C2-33525A4F8A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42ED0A9A-70CD-471D-AFE1-0F7371FE171B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="222">
   <si>
     <t>Totals</t>
   </si>
@@ -675,6 +675,33 @@
   </si>
   <si>
     <t>https://product.tdk.com/system/files/dam/doc/product/capacitor/ceramic/mlcc/catalog/mlcc_commercial_midvoltage_en.pdf</t>
+  </si>
+  <si>
+    <t>CL10B224KO8NNNC</t>
+  </si>
+  <si>
+    <t>1276-1112-1-ND</t>
+  </si>
+  <si>
+    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/920/CL10B224KO8NNNC_Spec.pdf</t>
+  </si>
+  <si>
+    <t>http://www.samsungsem.com/kr/support/product-search/mlcc/CL21B224KBFVPNE.jsp</t>
+  </si>
+  <si>
+    <t>1276-7012-1-ND</t>
+  </si>
+  <si>
+    <t>CL21B224KBFVPNE</t>
+  </si>
+  <si>
+    <t>CL31B224KBFNNNE</t>
+  </si>
+  <si>
+    <t>1276-1106-1-ND</t>
+  </si>
+  <si>
+    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/6941/CL31B224KBFNNN.pdf</t>
   </si>
 </sst>
 </file>
@@ -771,8 +798,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3238162E-29AF-4017-AC7C-5AC564956ED2}" name="Table1" displayName="Table1" ref="C6:T55" totalsRowShown="0">
-  <autoFilter ref="C6:T55" xr:uid="{3238162E-29AF-4017-AC7C-5AC564956ED2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3238162E-29AF-4017-AC7C-5AC564956ED2}" name="Table1" displayName="Table1" ref="C6:T58" totalsRowShown="0">
+  <autoFilter ref="C6:T58" xr:uid="{3238162E-29AF-4017-AC7C-5AC564956ED2}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C14:T51">
     <sortCondition ref="D6:D55"/>
   </sortState>
@@ -1095,75 +1122,75 @@
       </c>
       <c r="C2">
         <f t="shared" ref="C2:T2" si="0">COUNTA(C7:C10007)</f>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="L2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="Q2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="S2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="T2">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="AA2" t="s">
         <v>1</v>
@@ -1179,7 +1206,7 @@
       </c>
       <c r="AB3">
         <f>MAX(C2:R2)</f>
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.35">
@@ -1245,7 +1272,7 @@
       </c>
       <c r="AB4">
         <f>SUM(Y7:Y9999)</f>
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.35">
@@ -4858,13 +4885,220 @@
       </c>
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E56" s="2"/>
+      <c r="A56">
+        <v>50</v>
+      </c>
+      <c r="C56" t="str">
+        <f>_xlfn.CONCAT(D56,"F ",F56,"V ",E56," ",G56," ",I56," ",J56," ",R56)</f>
+        <v>220nF 16V 0603 X7R SMD MLCC  </v>
+      </c>
+      <c r="D56" t="s">
+        <v>71</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F56">
+        <v>16</v>
+      </c>
+      <c r="G56" t="s">
+        <v>33</v>
+      </c>
+      <c r="H56">
+        <v>10</v>
+      </c>
+      <c r="I56" t="s">
+        <v>28</v>
+      </c>
+      <c r="J56" t="s">
+        <v>29</v>
+      </c>
+      <c r="K56" t="s">
+        <v>53</v>
+      </c>
+      <c r="L56" t="s">
+        <v>213</v>
+      </c>
+      <c r="M56" t="s">
+        <v>37</v>
+      </c>
+      <c r="N56" t="s">
+        <v>214</v>
+      </c>
+      <c r="O56" t="s">
+        <v>215</v>
+      </c>
+      <c r="P56" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>41</v>
+      </c>
+      <c r="R56" t="s">
+        <v>42</v>
+      </c>
+      <c r="S56" t="b">
+        <v>0</v>
+      </c>
+      <c r="T56" t="b">
+        <v>1</v>
+      </c>
+      <c r="W56">
+        <f t="shared" ref="W56:W57" si="26">COUNTBLANK(C56:R56)</f>
+        <v>0</v>
+      </c>
+      <c r="X56">
+        <f t="shared" ref="X56:X57" si="27">100*COUNTA(C56:R56)/$AB$7</f>
+        <v>100</v>
+      </c>
+      <c r="Y56">
+        <f t="shared" ref="Y56:Y57" si="28">IF(X56=100,1,0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="57" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E57" s="2"/>
+      <c r="A57">
+        <v>51</v>
+      </c>
+      <c r="C57" t="str">
+        <f t="shared" ref="C57:C58" si="29">_xlfn.CONCAT(D57,"F ",F57,"V ",E57," ",G57," ",I57," ",J57," ",R57)</f>
+        <v>220nF 50V 0805 X7R SMD MLCC  </v>
+      </c>
+      <c r="D57" t="s">
+        <v>71</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F57">
+        <v>50</v>
+      </c>
+      <c r="G57" t="s">
+        <v>33</v>
+      </c>
+      <c r="H57">
+        <v>10</v>
+      </c>
+      <c r="I57" t="s">
+        <v>28</v>
+      </c>
+      <c r="J57" t="s">
+        <v>29</v>
+      </c>
+      <c r="K57" t="s">
+        <v>53</v>
+      </c>
+      <c r="L57" t="s">
+        <v>218</v>
+      </c>
+      <c r="M57" t="s">
+        <v>37</v>
+      </c>
+      <c r="N57" t="s">
+        <v>217</v>
+      </c>
+      <c r="O57" t="s">
+        <v>216</v>
+      </c>
+      <c r="P57" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>95</v>
+      </c>
+      <c r="R57" t="s">
+        <v>42</v>
+      </c>
+      <c r="S57" t="b">
+        <v>0</v>
+      </c>
+      <c r="T57" t="b">
+        <v>1</v>
+      </c>
+      <c r="W57">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="X57">
+        <f t="shared" si="27"/>
+        <v>100</v>
+      </c>
+      <c r="Y57">
+        <f t="shared" si="28"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="58" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="E58" s="2"/>
+      <c r="A58">
+        <v>52</v>
+      </c>
+      <c r="C58" t="str">
+        <f t="shared" si="29"/>
+        <v>220nF 50V 1206 X7R SMD MLCC  </v>
+      </c>
+      <c r="D58" t="s">
+        <v>71</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F58">
+        <v>50</v>
+      </c>
+      <c r="G58" t="s">
+        <v>33</v>
+      </c>
+      <c r="H58">
+        <v>10</v>
+      </c>
+      <c r="I58" t="s">
+        <v>28</v>
+      </c>
+      <c r="J58" t="s">
+        <v>29</v>
+      </c>
+      <c r="K58" t="s">
+        <v>53</v>
+      </c>
+      <c r="L58" t="s">
+        <v>219</v>
+      </c>
+      <c r="M58" t="s">
+        <v>37</v>
+      </c>
+      <c r="N58" t="s">
+        <v>220</v>
+      </c>
+      <c r="O58" t="s">
+        <v>221</v>
+      </c>
+      <c r="P58" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>52</v>
+      </c>
+      <c r="R58" t="s">
+        <v>42</v>
+      </c>
+      <c r="S58" t="b">
+        <v>0</v>
+      </c>
+      <c r="T58" t="b">
+        <v>1</v>
+      </c>
+      <c r="W58">
+        <f t="shared" ref="W58" si="30">COUNTBLANK(C58:R58)</f>
+        <v>0</v>
+      </c>
+      <c r="X58">
+        <f t="shared" ref="X58" si="31">100*COUNTA(C58:R58)/$AB$7</f>
+        <v>100</v>
+      </c>
+      <c r="Y58">
+        <f t="shared" ref="Y58" si="32">IF(X58=100,1,0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.35">
       <c r="E59" s="2"/>

</xml_diff>